<commit_message>
adding joins to consult and reports for Consult Manager Modul
</commit_message>
<xml_diff>
--- a/templates_formats/cronograma.xlsx
+++ b/templates_formats/cronograma.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-1875" yWindow="3930" windowWidth="15000" windowHeight="6555" activeTab="2"/>
+    <workbookView xWindow="-1875" yWindow="3930" windowWidth="15000" windowHeight="6555"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,9 +63,6 @@
     <t>EVALUACION I MOMENTO MATERIA PENDIENTE</t>
   </si>
   <si>
-    <t>SEMANA ANIVERSARIO 28 DE OCTUBRE</t>
-  </si>
-  <si>
     <t>ENTREGA DE NOTAS AL DEPARTAMENTO DE EVALUACION</t>
   </si>
   <si>
@@ -127,6 +124,9 @@
   </si>
   <si>
     <t>"NOMBRE MUNICIPIO","NOMBRE ESTADO"</t>
+  </si>
+  <si>
+    <t>SEMANA ANIVERSARIO NOMBRE INSTITUTO</t>
   </si>
 </sst>
 </file>
@@ -640,7 +640,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -653,7 +653,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -666,7 +666,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
@@ -679,7 +679,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
@@ -692,7 +692,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -798,43 +798,43 @@
     </row>
     <row r="19" spans="4:5" ht="30" x14ac:dyDescent="0.25">
       <c r="D19" s="9" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="E19" s="12"/>
     </row>
     <row r="20" spans="4:5" ht="30" x14ac:dyDescent="0.25">
       <c r="D20" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E20" s="12"/>
     </row>
     <row r="21" spans="4:5" ht="30" x14ac:dyDescent="0.25">
       <c r="D21" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E21" s="12"/>
     </row>
     <row r="22" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D22" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E22" s="12"/>
     </row>
     <row r="23" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D23" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E23" s="12"/>
     </row>
     <row r="24" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D24" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E24" s="12"/>
     </row>
     <row r="25" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D25" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E25" s="12"/>
     </row>
@@ -1012,7 +1012,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -1022,7 +1022,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -1033,7 +1033,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
@@ -1043,7 +1043,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
@@ -1053,7 +1053,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -1119,43 +1119,43 @@
     </row>
     <row r="14" spans="1:10" ht="105" x14ac:dyDescent="0.25">
       <c r="D14" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E14" s="12"/>
     </row>
     <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="D15" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E15" s="12"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D16" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E16" s="12"/>
     </row>
     <row r="17" spans="4:5" ht="45" x14ac:dyDescent="0.25">
       <c r="D17" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E17" s="12"/>
     </row>
     <row r="18" spans="4:5" ht="30" x14ac:dyDescent="0.25">
       <c r="D18" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E18" s="12"/>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D19" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E19" s="12"/>
     </row>
     <row r="20" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D20" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E20" s="12"/>
     </row>
@@ -1227,7 +1227,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -1237,7 +1237,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -1248,7 +1248,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
@@ -1258,7 +1258,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
@@ -1269,7 +1269,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -1335,55 +1335,55 @@
     </row>
     <row r="14" spans="1:10" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D14" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E14" s="11"/>
     </row>
     <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="D15" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="11"/>
     </row>
     <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="D16" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E16" s="11"/>
     </row>
     <row r="17" spans="4:5" ht="30" x14ac:dyDescent="0.25">
       <c r="D17" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E17" s="11"/>
     </row>
     <row r="18" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D18" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" s="11"/>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D19" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="4:5" ht="45" x14ac:dyDescent="0.25">
       <c r="D20" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D21" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D22" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E22" s="11"/>
     </row>

</xml_diff>